<commit_message>
Corregida compatibilidad de formulas de Excel para Google Sheets
</commit_message>
<xml_diff>
--- a/Proyecto_Estadistica_UMG.xlsx
+++ b/Proyecto_Estadistica_UMG.xlsx
@@ -471,7 +471,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="31" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="J4" s="6">
-        <f>CONTAR(E4:E33)</f>
+        <f>COUNT(E4:E33)</f>
         <v/>
       </c>
     </row>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="J5" s="5">
-        <f>PROMEDIO(E4:E33)</f>
+        <f>AVERAGE(E4:E33)</f>
         <v/>
       </c>
     </row>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="J6" s="5">
-        <f>MEDIANA(E4:E33)</f>
+        <f>MEDIAN(E4:E33)</f>
         <v/>
       </c>
     </row>
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="J7" s="5">
-        <f>MODA.UNO(E4:E33)</f>
+        <f>MODE.SNGL(E4:E33)</f>
         <v/>
       </c>
     </row>
@@ -867,7 +867,7 @@
         </is>
       </c>
       <c r="J12" s="5">
-        <f>DESVEST.M(E4:E33)</f>
+        <f>STDEV.S(E4:E33)</f>
         <v/>
       </c>
     </row>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="J14" s="5">
-        <f>CUARTIL.INC(E4:E33; 1)</f>
+        <f>QUARTILE.INC(E4:E33, 1)</f>
         <v/>
       </c>
     </row>
@@ -981,7 +981,7 @@
         </is>
       </c>
       <c r="J15" s="5">
-        <f>CUARTIL.INC(E4:E33; 2)</f>
+        <f>QUARTILE.INC(E4:E33, 2)</f>
         <v/>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="J16" s="5">
-        <f>CUARTIL.INC(E4:E33; 3)</f>
+        <f>QUARTILE.INC(E4:E33, 3)</f>
         <v/>
       </c>
     </row>

</xml_diff>